<commit_message>
Domain behaviour: count an axis only when the assigned value differs
A difference only in the value list is reported separately
(Axes_Value_List_Only). Evaluator is no longer an axis in RS, TR, TU;
position no longer shows as location in VS.

Observables_Direction: table from the new run, reading revised,
Step 1 reworded to read and record. README: the upstream step is
stated as later and separate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ACab21UkwTnWJ8Qq1ZztWj
</commit_message>
<xml_diff>
--- a/domain-behaviour/interim/Domain_Behaviour.xlsx
+++ b/domain-behaviour/interim/Domain_Behaviour.xlsx
@@ -23,16 +23,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -51,21 +48,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,77 +423,77 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Observation_Class</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Consumer_Class</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Consumer_Status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>BCs</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>DSSs</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>BCs_Fanning_Out</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Max_Fanout</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Primary_Axis</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Axes_Seen</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Scale_Mix</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Share_With_Units</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Share_With_Specimen</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Share_With_Method</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Share_With_Location</t>
         </is>
@@ -852,12 +840,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>location 1</t>
+          <t>(none) 1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1528,12 +1516,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>location 1</t>
+          <t>(none) 1</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1590,7 +1578,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>location 5; category 1</t>
+          <t>location 4; category 1</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1801,12 +1789,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>category; evaluator</t>
+          <t>category</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>category 4; evaluator 4</t>
+          <t>category 4</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -1956,12 +1944,12 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>category 3</t>
+          <t>(none) 3</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -2013,12 +2001,12 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>evaluator</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>evaluator 4</t>
+          <t>(none) 4</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -2132,7 +2120,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>(none) 3; evaluator 2</t>
+          <t>(none) 5</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -2241,12 +2229,12 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>location 4</t>
+          <t>(none) 4</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -2278,36 +2266,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F84"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>bc_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>bc_short_name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>DSS_Count</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Axes</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Axes_Value_List_Only</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
         <is>
           <t>DS_Codes</t>
         </is>
@@ -2337,7 +2330,8 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
         <is>
           <t>AE; AEPRESP</t>
         </is>
@@ -2367,7 +2361,8 @@
           <t>category</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
         <is>
           <t>CMFREE; CMPRESP; CMPRIORBREASTCANCER; CMPRIORCANCER</t>
         </is>
@@ -2394,10 +2389,15 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>location</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>EXPOSCOLL; EXPOSCOLL_XANOMELINEPLACEBO</t>
         </is>
@@ -2427,7 +2427,8 @@
           <t>method; test detail; scale</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
         <is>
           <t>TRNSCPTNFRAGCNT; TRNSCPTNGENTRNIND; TRNSCPTNNORMLVL; TRNSCPTNNORMLVLDIFF; TRNSCPTNPERCNTRANK</t>
         </is>
@@ -2457,7 +2458,8 @@
           <t>test detail</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
         <is>
           <t>CPNUMVARALTEXON; CPNUMVARATIO; CPNUMVARINTP; CPNUMVARNUMGCPY</t>
         </is>
@@ -2487,7 +2489,8 @@
           <t>method; test detail; scale</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
         <is>
           <t>SNVGENOTYPE; SNVPRAMACHG; SNVPRCSEQCHG; SNVREADEPTH; SNVVAREADEPTHRD; SNVVARIMPCLASS</t>
         </is>
@@ -2517,7 +2520,8 @@
           <t>test detail</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
         <is>
           <t>MICRISTBDETECT; MICRISTBOVRASTAT</t>
         </is>
@@ -2547,7 +2551,8 @@
           <t>test detail</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
         <is>
           <t>GENESIGINTP; GENESIGSCORE</t>
         </is>
@@ -2577,7 +2582,8 @@
           <t>test detail; scale</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
         <is>
           <t>SHRTVAREADEPTH; SHRTVAREADEPTHRD; SHRTVARIMPCLASS; SHRTVARPRAMACHG; SHRTVARPRCSEQCHG</t>
         </is>
@@ -2607,7 +2613,8 @@
           <t>specimen; method; test detail; scale</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
         <is>
           <t>TMBNORMNUMSEQVAR; TMBNUMSEQVAR; TMBVARSEQBURDINTP</t>
         </is>
@@ -2637,7 +2644,8 @@
           <t>test detail</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
         <is>
           <t>SEQREAREADDEPTH; SEQREARGENE1; SEQREARGENE2; SEQREARIMPCLASS; SEQREARPREINFRIND; SEQREARTYPE</t>
         </is>
@@ -2667,7 +2675,8 @@
           <t>method; test detail</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
         <is>
           <t>VNTRNCAGRPT; VNTRNUCLSEQ; VNTRPNCAGRPT</t>
         </is>
@@ -2697,7 +2706,8 @@
           <t>test detail</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
         <is>
           <t>VARPROFPRDIPLO; VARPROFPRPHENO</t>
         </is>
@@ -2727,7 +2737,8 @@
           <t>binding agent</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
         <is>
           <t>MBIGGABAA; MBIGGABAF; MBIGGABAV; MBIGGABBB; MBIGGABC; MBIGGABCD; MBIGGABCP; MBIGGABCTE; MBIGGABCTR; MBIGGABCTT; MBIGGABCV; MBIGGABDV; MBIGGABEBVCA; MBIGGABEBVEDA; MBIGGABEBVENA1; MBIGGABHAV; MBIGGABHBVCA; MBIGGABHDV; MBIGGABHEV; MBIGGABHHV1; MBIGGABHHV2; MBIGGABHP; MBIGGABHPVB19; MBIGGABHSV; MBIGGABIAV; MBIGGABIBV; MBIGGABLP; MBIGGABMBTC; MBIGGABMM; MBIGGABMPP; MBIGGABMRV; MBIGGABNGLI4; MBIGGABPC; MBIGGABRV; MBIGGABSARSCV2; MBIGGABSG; MBIGGABSP; MBIGGABSPDST1; MBIGGABSPDST10A; MBIGGABSPDST11A; MBIGGABSPDST12F; MBIGGABSPDST14; MBIGGABSPDST15B; MBIGGABSPDST17F; MBIGGABSPDST18C; MBIGGABSPDST19A; MBIGGABSPDST19F; MBIGGABSPDST2; MBIGGABSPDST20A; MBIGGABSPDST22F; MBIGGABSPDST23F; MBIGGABSPDST3; MBIGGABSPDST33F; MBIGGABSPDST4; MBIGGABSPDST5; MBIGGABSPDST6B; MBIGGABSPDST7F; MBIGGABSPDST8; MBIGGABSPDST9N; MBIGGABSPDST9V; MBIGGABTG; MBIGGABVCTBSU; MBIGGABVZV</t>
         </is>
@@ -2757,7 +2768,8 @@
           <t>specimen; method; binding agent; test detail; scale</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr">
         <is>
           <t>ARIGEABAA; ARIGEABAAMAST7; ARIGEABAARAST; ARIGEABACA; ARIGEABACARAST; ARIGEABAF; ARIGEABAFRAST; ARIGEABAHDMA; ARIGEABAHDMARAST; ARIGEABAHDMMAST7; ARIGEABAMA; ARIGEABAMARAST; ARIGEABAMAST7; ARIGEABBEP; ARIGEABBEPRAST; ARIGEABBGP; ARIGEABBGPRAST; ARIGEABBMAST7; ARIGEABBMAST72; ARIGEABBMVA; ARIGEABBMVARAST; ARIGEABCA; ARIGEABCANA; ARIGEABCANARAST; ARIGEABCARAST; ARIGEABCBMAST7; ARIGEABCDA; ARIGEABCDARAST; ARIGEABCDMAST7; ARIGEABCH; ARIGEABCHRAST; ARIGEABCMA; ARIGEABCMARAST; ARIGEABCMAST7; ARIGEABCMIXA; ARIGEABCMIXARAST; ARIGEABCMMAST7; ARIGEABCNA; ARIGEABCNARAST; ARIGEABCPMAST7; ARIGEABCRP; ARIGEABCRPRAST; ARIGEABDDA; ARIGEABDDARAST; ARIGEABDDMAST7; ARIGEABEHDMA; ARIGEABEHDMARAST; ARIGEABEPP; ARIGEABEPPRAST; ARIGEABEWA; ARIGEABEWARAST; ARIGEABEWMAST7; ARIGEABFP; ARIGEABFPRAST; ARIGEABGCA; ARIGEABGCARAST; ARIGEABGKMAST7; ARIGEABGMP; ARIGEABGMPRAST; ARIGEABHDMAST7; ARIGEABICMAST7; ARIGEABJAMAST7; ARIGEABJCMAST7; ARIGEABM; ARIGEABMA; ARIGEABMARAST; ARIGEABMMA; ARIGEABMMARAST; ARIGEABMMAST7; ARIGEABMMAST72; ARIGEABMR; ARIGEABMRAST; ARIGEABMRRAST; ARIGEABNMA; ARIGEABNMARAST; ARIGEABNRLMAST7; ARIGEABOGMAST7; ARIGEABOGP; ARIGEABOGPRAST; ARIGEABOMAST7; ARIGEABOTP; ARIGEABOTPRAST; ARIGEABPA; ARIGEABPARAST; ARIGEABPBMAST7; ARIGEABPC; ARIGEABPCRAST; ARIGEABPMAST7; ARIGEABPMAST72; ARIGEABPMAST73; ARIGEABRMAST7; ARIGEABRTP; ARIGEABRTPRAST; ARIGEABSA; ARIGEABSARAST; ARIGEABSBP; ARIGEABSBPRAST; ARIGEABSMA; ARIGEABSMARAST; ARIGEABSMAST7; ARIGEABSSMAST7; ARIGEABSSMAST72; ARIGEABTAA; ARIGEABTAARAST; ARIGEABTAMAST7; ARIGEABTAMAST72; ARIGEABTGMAST7; ARIGEABTGP; ARIGEABTGPRAST; ARIGEABTMAST7; ARIGEABTMP; ARIGEABTMPRAST; ARIGEABTSA; ARIGEABTSARAST; ARIGEABWA; ARIGEABWARAST; ARIGEABWBMAST7; ARIGEABWEP; ARIGEABWEPRAST; ARIGEABWMP; ARIGEABWMPMAST7; ARIGEABWMPRAST; ARIGEABWOP; ARIGEABWOPRAST; ARIGEABWRGP; ARIGEABWRGPRAST; ARIGEABWRP; ARIGEABWRPRAST</t>
         </is>
@@ -2787,7 +2799,8 @@
           <t>binding agent</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
         <is>
           <t>ARIGAABACA; ARIGAABALTERNARIA; ARIGAABBGP; ARIGAABCDA; ARIGAABDDA; ARIGAABEPP; ARIGAABGA; ARIGAABGCA; ARIGAABGMP; ARIGAABMMA; ARIGAABMUCOR; ARIGAABOGP; ARIGAABPENICILLUM; ARIGAABSBP; ARIGAABTGP; ARIGAABWMP; ARIGAABWRP</t>
         </is>
@@ -2817,7 +2830,8 @@
           <t>binding agent; test detail; scale</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
         <is>
           <t>ARIGGABAARAST; ARIGGABACA; ARIGGABACARAST; ARIGGABAFRAST; ARIGGABAHDMA; ARIGGABAHDMARAST; ARIGGABAMA; ARIGGABAMARAST; ARIGGABBGP; ARIGGABBGPRAST; ARIGGABBMVA; ARIGGABBMVARAST; ARIGGABCDA; ARIGGABCDARAST; ARIGGABCMA; ARIGGABCMARAST; ARIGGABDDA; ARIGGABDDARAST; ARIGGABDMA; ARIGGABDMARAST; ARIGGABEHDMA; ARIGGABEHDMARAST; ARIGGABEPP; ARIGGABEPPRAST; ARIGGABGA; ARIGGABGCA; ARIGGABGCARAST; ARIGGABGMP; ARIGGABGMPRAST; ARIGGABKLH; ARIGGABMMA; ARIGGABMMARAST; ARIGGABMR; ARIGGABMRPRAST; ARIGGABNMA; ARIGGABNMARAST; ARIGGABOGP; ARIGGABOGPRAST; ARIGGABPFRAST; ARIGGABSBP; ARIGGABSBPRAST; ARIGGABSMA; ARIGGABSMARAST; ARIGGABSTGPRAST; ARIGGABSTMPRAST; ARIGGABSWMPRAST; ARIGGABSWRPRAST; ARIGGABTGP; ARIGGABTMP; ARIGGABWEP; ARIGGABWEPRAST; ARIGGABWMP; ARIGGABWRP</t>
         </is>
@@ -2847,7 +2861,8 @@
           <t>binding agent; scale</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
         <is>
           <t>MBIMABA; MBIMABAPN; MBIMABBB; MBIMABBBPN; MBIMABCMV; MBIMABCMVPN; MBIMABCOCC; MBIMABCOCCPN; MBIMABCP; MBIMABCPPN; MBIMABCT; MBIMABCTPN; MBIMABDV; MBIMABDVPN; MBIMABEBVCA; MBIMABEBVCAPN; MBIMABEV; MBIMABEVPN; MBIMABHAV; MBIMABHAVPN; MBIMABHBVCA; MBIMABHBVCAPN; MBIMABHDV; MBIMABHDVPN; MBIMABHEV; MBIMABHEVPN; MBIMABHHV1; MBIMABHHV1PN; MBIMABHHV2; MBIMABHHV2PN; MBIMABHPB19; MBIMABHPB19PN; MBIMABHSV; MBIMABHSVPN; MBIMABLP; MBIMABLPPN; MBIMABMMV; MBIMABMMVPN; MBIMABMP; MBIMABMPPN; MBIMABMRV; MBIMABMRVPN; MBIMABNGLI4; MBIMABNGLI4PN; MBIMABRV; MBIMABRVPN; MBIMABSARSC2; MBIMABSARSC2PN; MBIMABTG; MBIMABTGPN; MBIMABVZV; MBIMABVZVPN</t>
         </is>
@@ -2877,7 +2892,8 @@
           <t>binding agent; scale</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
         <is>
           <t>ATIGMABB2G1; ATIGMABB2G1PN; ATIGMABC; ATIGMABCPN; ATIGMABLKMT1A; ATIGMABLKMT1APN; ATIGMABP; ATIGMABPL; ATIGMABPLPN; ATIGMABPPN; ATIGMABTT; ATIGMABTTPN</t>
         </is>
@@ -2907,7 +2923,8 @@
           <t>specimen; method; category; scale</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
         <is>
           <t>GLUCBLD; GLUCPE; GLUCPL; GLUCSER; GLUCSERPL; GLUCUA; GLUCURIN; GLUCURINPRES</t>
         </is>
@@ -2937,7 +2954,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
         <is>
           <t>CMONOXBLD; CMONOXEXPAIR</t>
         </is>
@@ -2967,7 +2985,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
         <is>
           <t>NICOTINESERPL; NICOTINEURIN</t>
         </is>
@@ -2997,7 +3016,8 @@
           <t>specimen; category; scale</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
         <is>
           <t>BILISERPL; BILIURIN; BILIURINPRES</t>
         </is>
@@ -3027,7 +3047,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
         <is>
           <t>APTTBLD; APTTPPP</t>
         </is>
@@ -3057,7 +3078,8 @@
           <t>specimen; method; category; scale</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
         <is>
           <t>RBCBLD; RBCURIN; RBCURINDIP; RBCURINPRES; RBCURINSEDPRES</t>
         </is>
@@ -3087,7 +3109,8 @@
           <t>specimen; method; category; scale</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
         <is>
           <t>WBCBLD; WBCURIN; WBCURINDIP; WBCURINPRES; WBCURINSEDPRES</t>
         </is>
@@ -3117,7 +3140,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
         <is>
           <t>PTBLD; PTPPP</t>
         </is>
@@ -3147,7 +3171,8 @@
           <t>specimen; category; scale</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
         <is>
           <t>ALBSERPL; ALBURIN; ALBURINPRES</t>
         </is>
@@ -3177,7 +3202,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
         <is>
           <t>CABLD; CASERPL</t>
         </is>
@@ -3207,7 +3233,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
         <is>
           <t>CKBLD; CKSERPL</t>
         </is>
@@ -3237,7 +3264,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
         <is>
           <t>CLBLD; CLSERPL</t>
         </is>
@@ -3267,7 +3295,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
         <is>
           <t>CO2BLD; CO2SERPL</t>
         </is>
@@ -3297,7 +3326,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
         <is>
           <t>CREATSERPL; CREATURIN</t>
         </is>
@@ -3327,7 +3357,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
         <is>
           <t>INRBLD; INRPPP</t>
         </is>
@@ -3357,7 +3388,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
         <is>
           <t>SODIUMBLD; SODIUMSERPL; SODIUMURIN</t>
         </is>
@@ -3387,7 +3419,8 @@
           <t>scale</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
         <is>
           <t>NITRITEURIN; NITRITEURINPRES; UROBILURINPRES</t>
         </is>
@@ -3417,7 +3450,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
         <is>
           <t>TSHBLD; TSHSERPL</t>
         </is>
@@ -3447,7 +3481,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
         <is>
           <t>VITB12BLD; VITB12SERPL</t>
         </is>
@@ -3477,7 +3512,8 @@
           <t>specimen; category</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr">
         <is>
           <t>MACROCYBLD; MACROCYURNSED</t>
         </is>
@@ -3507,7 +3543,8 @@
           <t>specimen; category</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
         <is>
           <t>MICROCYBLD; MICROCYURN; MICROCYURNSED</t>
         </is>
@@ -3537,7 +3574,8 @@
           <t>method</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
         <is>
           <t>HGBBLD; HGBBLDDIP</t>
         </is>
@@ -3567,7 +3605,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr">
         <is>
           <t>HCGSERPL; HCGURIN</t>
         </is>
@@ -3597,7 +3636,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
         <is>
           <t>KBLD; KSERPL; KURIN</t>
         </is>
@@ -3627,7 +3667,8 @@
           <t>scale</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
         <is>
           <t>KETONESURIN; KETONESURINPRES</t>
         </is>
@@ -3657,7 +3698,8 @@
           <t>specimen; category; scale</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
         <is>
           <t>PROTSERPL; PROTURIN; PROTURINPRES</t>
         </is>
@@ -3687,7 +3729,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
         <is>
           <t>VITB9BLD; VITB9SERPL</t>
         </is>
@@ -3717,7 +3760,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
         <is>
           <t>OCCBLDSTOOL; OCCBLDURINPRES</t>
         </is>
@@ -3747,7 +3791,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
         <is>
           <t>TROPONIBLD; TROPONISERPL</t>
         </is>
@@ -3777,7 +3822,8 @@
           <t>specimen</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
         <is>
           <t>CYSTATCSERPL; CYSTATCURIN</t>
         </is>
@@ -3807,7 +3853,8 @@
           <t>test detail; scale</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
         <is>
           <t>HCRNASERPL; HCRNASERPLPRES</t>
         </is>
@@ -3837,7 +3884,8 @@
           <t>test detail; scale</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
         <is>
           <t>HBCAGSERPL; HBCAGSERPLPRES</t>
         </is>
@@ -3867,7 +3915,8 @@
           <t>test detail; scale</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
         <is>
           <t>SAR2RNAQNTCYC; SAR2RNAVIRAL</t>
         </is>
@@ -3897,7 +3946,8 @@
           <t>test detail; scale</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
         <is>
           <t>HBSAGSERPL; HBSAGSERPLPRES</t>
         </is>
@@ -3927,7 +3977,8 @@
           <t>category</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr">
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
         <is>
           <t>MEDHISTFREE; MEDHISTPRESP; MHALZHEIMERS; MHBRCADIAG; MHBRCARELAPSE; MHCONFUSIONALEPISODES; MHESSENTIALTREMOR; MHESSENTIALTREMOREXPYR; MHEXTRAPYRAMIDAL; MHFACIALMASKING; MHRIGIDITYUPPEREXTREMITY; MHSENSITIVITYNEUROLEPTICS; MHVISUALHALLUCINATIONS</t>
         </is>
@@ -3957,7 +4008,8 @@
           <t>test detail</t>
         </is>
       </c>
-      <c r="F56" t="inlineStr">
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
         <is>
           <t>ESTRCPTAPRPSCORE; ESTRCPTASINTSCORE; ESTRCPTATOTSCORE</t>
         </is>
@@ -3987,7 +4039,8 @@
           <t>test detail</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
         <is>
           <t>PROGESTRAPRPSCORE; PROGESTRASINTSCORE; PROGESTRATOTSCORE</t>
         </is>
@@ -4014,10 +4067,15 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
           <t>location</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="G58" t="inlineStr">
         <is>
           <t>SGJSNSCRFJ; SGJSNSCRHW</t>
         </is>
@@ -4044,10 +4102,15 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>location; category</t>
+          <t>category</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
         <is>
           <t>RADIATIONCANCER; RADTHERAPHYBREASTCANCER</t>
         </is>
@@ -4077,7 +4140,8 @@
           <t>location</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
         <is>
           <t>MRI; MRIBRAIN</t>
         </is>
@@ -4107,7 +4171,8 @@
           <t>location</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
         <is>
           <t>CTSCAN; CTSCANABDOMIN; CTSCANCHEST; CTSCANPELVIS</t>
         </is>
@@ -4137,7 +4202,8 @@
           <t>location</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
         <is>
           <t>XRAY; XRAYCHEST</t>
         </is>
@@ -4167,7 +4233,8 @@
           <t>location</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
         <is>
           <t>SCINTIGRAPHY; SCINTIGRAPHYBONE</t>
         </is>
@@ -4194,10 +4261,15 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>category; evaluator</t>
+          <t>category</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
+        <is>
+          <t>evaluator</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
         <is>
           <t>NEWLIND_LUGANO; NEWLIND_RANO</t>
         </is>
@@ -4224,10 +4296,15 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>category; evaluator</t>
+          <t>category</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
+        <is>
+          <t>evaluator</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
         <is>
           <t>TRGRESP; TRGRESP_LUGANO; TRGRESP_RANO</t>
         </is>
@@ -4254,10 +4331,15 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>category; evaluator</t>
+          <t>category</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
+        <is>
+          <t>evaluator</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
         <is>
           <t>NTRGRESP; NTRGRESP_LUGANO</t>
         </is>
@@ -4284,10 +4366,15 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>category; evaluator</t>
+          <t>category</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
+        <is>
+          <t>evaluator</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
         <is>
           <t>OVRLRESP; OVRLRESP_LUGANO; OVRLRESP_RANO</t>
         </is>
@@ -4314,10 +4401,15 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="G68" t="inlineStr">
         <is>
           <t>CIGARETTEHX; CIGARHX; PIPEHX; TOBACCOHX</t>
         </is>
@@ -4344,10 +4436,15 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F69" t="inlineStr">
+      <c r="G69" t="inlineStr">
         <is>
           <t>CAFFEINEHX; COFFEEHX; COLAHX; TEAHIX</t>
         </is>
@@ -4374,10 +4471,15 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>ALCOHOLHX; BEERHX; DISTILLEDSPIRITSHX; WINEHX</t>
         </is>
@@ -4404,10 +4506,15 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
           <t>evaluator</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="G71" t="inlineStr">
         <is>
           <t>LNSTATE; LNSTATE_RECIST1_1</t>
         </is>
@@ -4434,10 +4541,15 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
           <t>evaluator</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="G72" t="inlineStr">
         <is>
           <t>NEW_TUMSTATE_RECIST1_1; NONNODAL_TUMSTATE_RECIST1_1; TUMSTATE</t>
         </is>
@@ -4464,10 +4576,15 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
           <t>evaluator</t>
         </is>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="G73" t="inlineStr">
         <is>
           <t>LDIAM; LDIAM_RECIST1_1</t>
         </is>
@@ -4494,10 +4611,15 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
           <t>evaluator</t>
         </is>
       </c>
-      <c r="F74" t="inlineStr">
+      <c r="G74" t="inlineStr">
         <is>
           <t>LPERP; LPERP_RECIST1_1</t>
         </is>
@@ -4527,7 +4649,8 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
         <is>
           <t>EGRDMETH; HEGRDMTH</t>
         </is>
@@ -4554,10 +4677,15 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
           <t>evaluator</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="G76" t="inlineStr">
         <is>
           <t>NTIND; NTIND_RECIST1_1</t>
         </is>
@@ -4584,10 +4712,15 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
           <t>evaluator</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr">
+      <c r="G77" t="inlineStr">
         <is>
           <t>TIND; TIND_RECIST1_1</t>
         </is>
@@ -4617,7 +4750,8 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr">
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
         <is>
           <t>TUMERGE; TUMERGE_RECIST1_1</t>
         </is>
@@ -4647,7 +4781,8 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="F79" t="inlineStr">
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
         <is>
           <t>TUSPLIT; TUSPLIT_RECIST1_1</t>
         </is>
@@ -4677,7 +4812,8 @@
           <t>(none)</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr">
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
         <is>
           <t>TUMIDENT; TUMIDENT_RECIST1_1</t>
         </is>
@@ -4704,10 +4840,15 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
           <t>location</t>
         </is>
       </c>
-      <c r="F81" t="inlineStr">
+      <c r="G81" t="inlineStr">
         <is>
           <t>SYSBP; SYSBP_EXT</t>
         </is>
@@ -4734,10 +4875,15 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
           <t>location</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr">
+      <c r="G82" t="inlineStr">
         <is>
           <t>DIABP; DIABP_EXT</t>
         </is>
@@ -4764,10 +4910,15 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
           <t>location</t>
         </is>
       </c>
-      <c r="F83" t="inlineStr">
+      <c r="G83" t="inlineStr">
         <is>
           <t>PULSE; PULSE_EXT</t>
         </is>
@@ -4794,10 +4945,15 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
+          <t>(none)</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
           <t>location</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="G84" t="inlineStr">
         <is>
           <t>HR; HR_EXT</t>
         </is>
@@ -4818,32 +4974,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Result_Scales</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>DSSs</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>With_Units</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Without_Units</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Flag</t>
         </is>
@@ -6756,42 +6912,42 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Consumer</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Claim_ID</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Claim</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Holds</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Evidence</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
@@ -7022,77 +7178,77 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>domain</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Observation_Class</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Consumer_Class</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Consumer_Status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>BCs</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>DSSs</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>BCs_Fanning_Out</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Max_Fanout</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Primary_Axis</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Axes_Seen</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Scale_Mix</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Share_With_Units</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Share_With_Specimen</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Share_With_Method</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Share_With_Location</t>
         </is>
@@ -7439,12 +7595,12 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>location 1</t>
+          <t>(none) 1</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -7705,7 +7861,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>location 5; category 1</t>
+          <t>location 4; category 1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -7904,12 +8060,12 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>category 3</t>
+          <t>(none) 3</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -7961,12 +8117,12 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>evaluator</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>evaluator 4</t>
+          <t>(none) 4</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -8080,7 +8236,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>(none) 3; evaluator 2</t>
+          <t>(none) 5</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -8116,12 +8272,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>measure</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
@@ -8467,7 +8623,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>(none)</t>
         </is>
       </c>
     </row>
@@ -8879,7 +9035,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>(none)</t>
         </is>
       </c>
     </row>
@@ -9047,7 +9203,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>category; evaluator</t>
+          <t>category</t>
         </is>
       </c>
     </row>
@@ -9147,7 +9303,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>(none)</t>
         </is>
       </c>
     </row>
@@ -9183,7 +9339,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>evaluator</t>
+          <t>(none)</t>
         </is>
       </c>
     </row>
@@ -9323,7 +9479,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>(none)</t>
         </is>
       </c>
     </row>
@@ -9402,12 +9558,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>pin</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>value</t>
         </is>

</xml_diff>